<commit_message>
adicao da verificacao de notas canceladas
</commit_message>
<xml_diff>
--- a/relatorio_financeiro.xlsx
+++ b/relatorio_financeiro.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F86"/>
+  <dimension ref="A1:F88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -471,17 +471,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>28/05/2025</t>
+          <t>29/05/2025</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0015-00</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2354</t>
+          <t>2356</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -489,7 +489,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>27/07/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -501,17 +501,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>28/05/2025</t>
+          <t>29/05/2025</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0015-00</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2353</t>
+          <t>2355</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -519,7 +519,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>27/07/2025</t>
+          <t>28/06/2025</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -531,17 +531,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>27/05/2025</t>
+          <t>28/05/2025</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0015-00</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2352</t>
+          <t>2354</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -549,7 +549,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>26/07/2025</t>
+          <t>27/06/2025</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -561,17 +561,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>22/05/2025</t>
+          <t>28/05/2025</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0015-00</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2351</t>
+          <t>2353</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -579,7 +579,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>27/06/2025</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -591,67 +591,67 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>14/01/2025</t>
+          <t>27/05/2025</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Não definido</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2315</t>
+          <t>2352</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>57857.44</v>
+        <v>77758.60000000001</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>26/06/2025</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>05/03/2025</t>
+          <t>Não definido</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>10/01/2025</t>
+          <t>22/05/2025</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Não definido</t>
+          <t>0014-00</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2314</t>
+          <t>2351</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>57857.44</v>
+        <v>77758.60000000001</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>17/02/2025</t>
+          <t>Não definido</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03/01/2025</t>
+          <t>14/01/2025</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -661,7 +661,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2311</t>
+          <t>2315</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -669,19 +669,19 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>17/02/2025</t>
+          <t>05/03/2025</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>17/12/2024</t>
+          <t>10/01/2025</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2310</t>
+          <t>2314</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -699,19 +699,19 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>14/02/2025</t>
+          <t>17/02/2025</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>13/12/2024</t>
+          <t>03/01/2025</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -721,7 +721,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2308</t>
+          <t>2311</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -729,19 +729,19 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>10/02/2025</t>
+          <t>17/02/2025</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>11/12/2024</t>
+          <t>17/12/2024</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -751,27 +751,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2306</t>
+          <t>2310</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>210421.33</v>
+        <v>57857.44</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>10/01/2025</t>
+          <t>14/02/2025</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>11/12/2024</t>
+          <t>13/12/2024</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2307</t>
+          <t>2308</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -789,7 +789,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -801,7 +801,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>09/12/2024</t>
+          <t>11/12/2024</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -811,27 +811,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2305</t>
+          <t>2306</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>28928.72</v>
+        <v>210421.33</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>10/02/2025</t>
+          <t>10/01/2025</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>09/12/2024</t>
+          <t>11/12/2024</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -841,15 +841,15 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2302</t>
+          <t>2307</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>28928.72</v>
+        <v>57857.44</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -861,7 +861,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06/12/2024</t>
+          <t>09/12/2024</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -871,27 +871,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2301</t>
+          <t>2305</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>115714.88</v>
+        <v>28928.72</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>17/03/2025</t>
+          <t>10/02/2025</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>02/12/2024</t>
+          <t>09/12/2024</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -901,27 +901,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2292</t>
+          <t>2302</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>130179.24</v>
+        <v>28928.72</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>03/02/2025</t>
+          <t>10/02/2025</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>19/11/2024</t>
+          <t>06/12/2024</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -931,27 +931,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2286</t>
+          <t>2301</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>130179.24</v>
+        <v>115714.88</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>24/01/2025</t>
+          <t>17/03/2025</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>18/11/2024</t>
+          <t>02/12/2024</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -961,7 +961,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2284</t>
+          <t>2292</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -969,19 +969,19 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>21/01/2025</t>
+          <t>03/02/2025</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>13/11/2024</t>
+          <t>19/11/2024</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2282</t>
+          <t>2286</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -999,19 +999,19 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>21/01/2025</t>
+          <t>24/01/2025</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>12/11/2024</t>
+          <t>18/11/2024</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1021,7 +1021,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2281</t>
+          <t>2284</t>
         </is>
       </c>
       <c r="D20" t="n">
@@ -1029,19 +1029,19 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>13/01/2025</t>
+          <t>21/01/2025</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>11/11/2024</t>
+          <t>13/11/2024</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1051,7 +1051,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2282</t>
         </is>
       </c>
       <c r="D21" t="n">
@@ -1059,19 +1059,19 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>13/01/2025</t>
+          <t>21/01/2025</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08/07/2024</t>
+          <t>12/11/2024</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1081,27 +1081,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2239</t>
+          <t>2281</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>51369.49</v>
+        <v>130179.24</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>09/09/2024</t>
+          <t>13/01/2025</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>26/06/2024</t>
+          <t>11/11/2024</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1111,27 +1111,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2235</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>51369.49</v>
+        <v>130179.24</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>28/08/2024</t>
+          <t>13/01/2025</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>25/06/2024</t>
+          <t>08/07/2024</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2234</t>
+          <t>2239</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1149,19 +1149,19 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Não definido</t>
+          <t>09/09/2024</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>25/06/2024</t>
+          <t>26/06/2024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2233</t>
+          <t>2235</t>
         </is>
       </c>
       <c r="D25" t="n">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1191,7 +1191,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>24/06/2024</t>
+          <t>25/06/2024</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1201,27 +1201,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2232</t>
+          <t>2234</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>102738.98</v>
+        <v>51369.49</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>28/08/2024</t>
+          <t>Não definido</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>24/06/2024</t>
+          <t>25/06/2024</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1231,7 +1231,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2231</t>
+          <t>2233</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1251,7 +1251,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>21/06/2024</t>
+          <t>24/06/2024</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2230</t>
+          <t>2232</t>
         </is>
       </c>
       <c r="D28" t="n">
@@ -1269,19 +1269,19 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>23/08/2024</t>
+          <t>28/08/2024</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>21/06/2024</t>
+          <t>24/06/2024</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1291,27 +1291,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>2229</t>
+          <t>2231</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>102738.98</v>
+        <v>51369.49</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>23/08/2024</t>
+          <t>28/08/2024</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>17/06/2024</t>
+          <t>21/06/2024</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1321,7 +1321,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2227</t>
+          <t>2230</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -1329,19 +1329,19 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>19/08/2024</t>
+          <t>23/08/2024</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>17/06/2024</t>
+          <t>21/06/2024</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1351,7 +1351,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2226</t>
+          <t>2229</t>
         </is>
       </c>
       <c r="D31" t="n">
@@ -1359,19 +1359,19 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>19/08/2024</t>
+          <t>23/08/2024</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>14/06/2024</t>
+          <t>17/06/2024</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1381,7 +1381,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2225</t>
+          <t>2227</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1401,7 +1401,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>12/06/2024</t>
+          <t>17/06/2024</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1411,7 +1411,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2224</t>
+          <t>2226</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1419,7 +1419,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1431,7 +1431,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>14/06/2024</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1441,7 +1441,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2225</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1449,19 +1449,19 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>16/08/2024</t>
+          <t>19/08/2024</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>11/06/2024</t>
+          <t>12/06/2024</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1471,7 +1471,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2221</t>
+          <t>2224</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1479,19 +1479,19 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>16/08/2024</t>
+          <t>19/08/2024</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>10/06/2024</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1501,7 +1501,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2220</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D36" t="n">
@@ -1509,19 +1509,19 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>09/08/2024</t>
+          <t>16/08/2024</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07/06/2024</t>
+          <t>11/06/2024</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1531,7 +1531,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2219</t>
+          <t>2221</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1539,19 +1539,19 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>13/08/2024</t>
+          <t>16/08/2024</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>06/06/2024</t>
+          <t>10/06/2024</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1561,7 +1561,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2216</t>
+          <t>2220</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -1569,19 +1569,19 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>13/08/2024</t>
+          <t>09/08/2024</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>06/06/2024</t>
+          <t>07/06/2024</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1591,7 +1591,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2215</t>
+          <t>2219</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -1599,7 +1599,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1621,7 +1621,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2214</t>
+          <t>2216</t>
         </is>
       </c>
       <c r="D40" t="n">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -1641,7 +1641,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>23/05/2024</t>
+          <t>06/06/2024</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2207</t>
+          <t>2215</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -1659,19 +1659,19 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Não definido</t>
+          <t>13/08/2024</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>23/05/2024</t>
+          <t>06/06/2024</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1681,7 +1681,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2206</t>
+          <t>2214</t>
         </is>
       </c>
       <c r="D42" t="n">
@@ -1689,19 +1689,19 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>22/07/2024</t>
+          <t>13/08/2024</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>21/05/2024</t>
+          <t>23/05/2024</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1711,7 +1711,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2204</t>
+          <t>2207</t>
         </is>
       </c>
       <c r="D43" t="n">
@@ -1719,19 +1719,19 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>22/07/2024</t>
+          <t>Não definido</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>21/05/2024</t>
+          <t>23/05/2024</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2205</t>
+          <t>2206</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -1761,7 +1761,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>20/05/2024</t>
+          <t>21/05/2024</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1771,7 +1771,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2199</t>
+          <t>2204</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1779,7 +1779,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -1791,7 +1791,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>17/05/2024</t>
+          <t>21/05/2024</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1801,7 +1801,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2197</t>
+          <t>2205</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1821,7 +1821,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>15/05/2024</t>
+          <t>20/05/2024</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1831,7 +1831,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>2199</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -1851,7 +1851,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>15/05/2024</t>
+          <t>17/05/2024</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2194</t>
+          <t>2197</t>
         </is>
       </c>
       <c r="D48" t="n">
@@ -1869,7 +1869,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1881,7 +1881,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>13/05/2024</t>
+          <t>15/05/2024</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2193</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -1899,19 +1899,19 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>15/07/2024</t>
+          <t>22/07/2024</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>13/05/2024</t>
+          <t>15/05/2024</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1921,7 +1921,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2192</t>
+          <t>2194</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -1929,19 +1929,19 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>15/07/2024</t>
+          <t>22/07/2024</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>10/05/2024</t>
+          <t>13/05/2024</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>2190</t>
+          <t>2193</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -1959,19 +1959,19 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>29/07/2024</t>
+          <t>15/07/2024</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>13/05/2024</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2185</t>
+          <t>2192</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -1989,19 +1989,19 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>05/07/2024</t>
+          <t>15/07/2024</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>02/05/2024</t>
+          <t>10/05/2024</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2011,7 +2011,7 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>2184</t>
+          <t>2190</t>
         </is>
       </c>
       <c r="D53" t="n">
@@ -2019,19 +2019,19 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>05/07/2024</t>
+          <t>29/07/2024</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>30/04/2024</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2183</t>
+          <t>2185</t>
         </is>
       </c>
       <c r="D54" t="n">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2061,7 +2061,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>25/04/2024</t>
+          <t>02/05/2024</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>2181</t>
+          <t>2184</t>
         </is>
       </c>
       <c r="D55" t="n">
@@ -2079,19 +2079,19 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>01/07/2024</t>
+          <t>05/07/2024</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>30/04/2024</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2180</t>
+          <t>2183</t>
         </is>
       </c>
       <c r="D56" t="n">
@@ -2109,19 +2109,19 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>25/06/2024</t>
+          <t>05/07/2024</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>24/04/2024</t>
+          <t>25/04/2024</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2131,7 +2131,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2179</t>
+          <t>2181</t>
         </is>
       </c>
       <c r="D57" t="n">
@@ -2139,19 +2139,19 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>25/06/2024</t>
+          <t>01/07/2024</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>23/04/2024</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2161,7 +2161,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2178</t>
+          <t>2179</t>
         </is>
       </c>
       <c r="D58" t="n">
@@ -2169,7 +2169,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2181,7 +2181,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>22/04/2024</t>
+          <t>24/04/2024</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2191,7 +2191,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2177</t>
+          <t>2180</t>
         </is>
       </c>
       <c r="D59" t="n">
@@ -2199,19 +2199,19 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>24/06/2024</t>
+          <t>25/06/2024</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>18/04/2024</t>
+          <t>23/04/2024</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2221,7 +2221,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>2176</t>
+          <t>2178</t>
         </is>
       </c>
       <c r="D60" t="n">
@@ -2229,19 +2229,19 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>24/06/2024</t>
+          <t>25/06/2024</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>17/04/2024</t>
+          <t>22/04/2024</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2251,7 +2251,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>2175</t>
+          <t>2177</t>
         </is>
       </c>
       <c r="D61" t="n">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2271,7 +2271,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>31/01/2024</t>
+          <t>18/04/2024</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2281,27 +2281,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>2161</t>
+          <t>2176</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>91292.95</v>
+        <v>102738.98</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Não definido</t>
+          <t>24/06/2024</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>25/01/2024</t>
+          <t>17/04/2024</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2311,27 +2311,27 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2156</t>
+          <t>2175</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>91292.95</v>
+        <v>102738.98</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>01/04/2024</t>
+          <t>24/06/2024</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>25/01/2024</t>
+          <t>31/01/2024</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2341,7 +2341,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>2155</t>
+          <t>2161</t>
         </is>
       </c>
       <c r="D64" t="n">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2379,7 +2379,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2391,7 +2391,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>19/01/2024</t>
+          <t>25/01/2024</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>2154</t>
+          <t>2156</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2409,7 +2409,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2421,7 +2421,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>19/01/2024</t>
+          <t>25/01/2024</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2153</t>
+          <t>2155</t>
         </is>
       </c>
       <c r="D67" t="n">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>01/04/2024</t>
+          <t>Não definido</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2469,7 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2481,7 +2481,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>17/01/2024</t>
+          <t>19/01/2024</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2491,27 +2491,27 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2149</t>
+          <t>2154</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>73034.36</v>
+        <v>91292.95</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>25/03/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>17/01/2024</t>
+          <t>19/01/2024</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2148</t>
+          <t>2153</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -2529,19 +2529,19 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>25/03/2024</t>
+          <t>01/04/2024</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>12/01/2024</t>
+          <t>17/01/2024</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2147</t>
+          <t>2148</t>
         </is>
       </c>
       <c r="D71" t="n">
@@ -2559,7 +2559,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -2571,7 +2571,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>12/01/2024</t>
+          <t>17/01/2024</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2581,7 +2581,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>2146</t>
+          <t>2149</t>
         </is>
       </c>
       <c r="D72" t="n">
@@ -2589,12 +2589,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>18/03/2024</t>
+          <t>25/03/2024</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2145</t>
+          <t>2147</t>
         </is>
       </c>
       <c r="D73" t="n">
@@ -2619,7 +2619,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2641,27 +2641,27 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>2144</t>
+          <t>2146</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>91292.95</v>
+        <v>73034.36</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>19/03/2024</t>
+          <t>18/03/2024</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>11/01/2024</t>
+          <t>12/01/2024</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2671,7 +2671,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2139</t>
+          <t>2145</t>
         </is>
       </c>
       <c r="D75" t="n">
@@ -2679,19 +2679,19 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>18/03/2024</t>
+          <t>25/03/2024</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>11/01/2024</t>
+          <t>12/01/2024</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2701,20 +2701,20 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2140</t>
+          <t>2144</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>73034.36</v>
+        <v>91292.95</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>18/03/2024</t>
+          <t>19/03/2024</t>
         </is>
       </c>
     </row>
@@ -2731,15 +2731,15 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>2141</t>
+          <t>2140</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>91292.95</v>
+        <v>73034.36</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -2751,7 +2751,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>10/01/2024</t>
+          <t>11/01/2024</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2761,7 +2761,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2138</t>
+          <t>2139</t>
         </is>
       </c>
       <c r="D78" t="n">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -2781,7 +2781,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>08/01/2024</t>
+          <t>11/01/2024</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2791,27 +2791,27 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2136</t>
+          <t>2141</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>73034.36</v>
+        <v>91292.95</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>12/03/2024</t>
+          <t>18/03/2024</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>08/01/2024</t>
+          <t>10/01/2024</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>2135</t>
+          <t>2138</t>
         </is>
       </c>
       <c r="D80" t="n">
@@ -2829,19 +2829,19 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>12/03/2024</t>
+          <t>18/03/2024</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>05/01/2024</t>
+          <t>08/01/2024</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2851,15 +2851,15 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>2134</t>
+          <t>2136</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>91292.95</v>
+        <v>73034.36</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -2871,7 +2871,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>02/01/2024</t>
+          <t>08/01/2024</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2881,7 +2881,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2132</t>
+          <t>2135</t>
         </is>
       </c>
       <c r="D82" t="n">
@@ -2889,7 +2889,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -2901,7 +2901,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>02/01/2024</t>
+          <t>05/01/2024</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2911,20 +2911,20 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2131</t>
+          <t>2134</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>73034.36</v>
+        <v>91292.95</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>19/02/2024</t>
+          <t>12/03/2024</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2132</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2949,7 +2949,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -2971,20 +2971,20 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>2129</t>
+          <t>2131</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>109551.54</v>
+        <v>73034.36</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>08/03/2024</t>
+          <t>19/02/2024</t>
         </is>
       </c>
     </row>
@@ -3001,7 +3001,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>2128</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D86" t="n">
@@ -3009,10 +3009,70 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>21/07/2025</t>
+          <t>21/06/2025</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
+        <is>
+          <t>12/03/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>02/01/2024</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Não definido</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2129</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>109551.54</v>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>21/06/2025</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>08/03/2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>02/01/2024</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Não definido</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2128</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>91292.95</v>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>21/06/2025</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
         <is>
           <t>08/03/2024</t>
         </is>

</xml_diff>